<commit_message>
Se ha creado y probado la funcion de merma tanto para gestion plus como para la apk Pos Movil
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BDCD59-01CF-4044-8236-65A2BEEE21BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A293CDF-F465-49B2-A315-E9FAF627A9E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pendientes" sheetId="4" r:id="rId1"/>
-    <sheet name="Merma" sheetId="5" r:id="rId2"/>
-    <sheet name="Productos" sheetId="1" r:id="rId3"/>
+    <sheet name="Productos" sheetId="1" r:id="rId2"/>
+    <sheet name="Merma" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>Código</t>
   </si>
@@ -272,6 +272,9 @@
   </si>
   <si>
     <t>Codigo</t>
+  </si>
+  <si>
+    <t>Nombre</t>
   </si>
   <si>
     <t>Cantidad</t>
@@ -441,18 +444,6 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EF2C0438-9E4A-4627-9C7E-7F5E94980D77}" name="Tabla3" displayName="Tabla3" ref="A1:C2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:C2" xr:uid="{EF2C0438-9E4A-4627-9C7E-7F5E94980D77}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{C072D279-60E7-4A77-A181-7342C511CC10}" name="Codigo"/>
-    <tableColumn id="2" xr3:uid="{F5A3544D-81FA-4776-91FB-8B4382A395DE}" name="Producto"/>
-    <tableColumn id="3" xr3:uid="{AEF872AD-16D2-4B3F-83A0-7DE864D77F35}" name="Cantidad"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F16977D9-4AF0-4513-B527-4EA8B61A33F3}" name="ALMACEN" displayName="ALMACEN" ref="A1:D33" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4" headerRowCellStyle="Énfasis5">
   <autoFilter ref="A1:D33" xr:uid="{F16977D9-4AF0-4513-B527-4EA8B61A33F3}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -467,6 +458,18 @@
     <tableColumn id="4" xr3:uid="{057FA4B9-0A24-4B11-AABE-D0F0F2217832}" name="Precio" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C2CB94C0-D619-434A-A4B0-0D891E997B38}" name="Tabla3" displayName="Tabla3" ref="A1:C2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:C2" xr:uid="{C2CB94C0-D619-434A-A4B0-0D891E997B38}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{F6BD4EA0-F565-4D2F-ADA2-8BC99D6A95A4}" name="Codigo"/>
+    <tableColumn id="2" xr3:uid="{5A4E880C-CBFA-4386-ADF7-91899EDE0D07}" name="Nombre"/>
+    <tableColumn id="3" xr3:uid="{BDD438F1-0115-4245-A313-92BAFF363974}" name="Cantidad"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -802,31 +805,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5F13078-3FF6-41B5-963F-89FAF9E936C4}">
-  <sheetPr codeName="Hoja3"/>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
   <dimension ref="A1:D32"/>
@@ -860,7 +838,7 @@
         <v>46</v>
       </c>
       <c r="C2" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D2" s="1">
         <v>600</v>
@@ -888,7 +866,7 @@
         <v>48</v>
       </c>
       <c r="C4" s="1">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="D4" s="1">
         <v>10</v>
@@ -902,7 +880,7 @@
         <v>49</v>
       </c>
       <c r="C5" s="1">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="D5" s="1">
         <v>300</v>
@@ -916,7 +894,7 @@
         <v>50</v>
       </c>
       <c r="C6" s="1">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="D6" s="1">
         <v>10</v>
@@ -930,7 +908,7 @@
         <v>52</v>
       </c>
       <c r="C7" s="1">
-        <v>16.489999999999998</v>
+        <v>12.489999999999998</v>
       </c>
       <c r="D7" s="1">
         <v>700</v>
@@ -958,7 +936,7 @@
         <v>54</v>
       </c>
       <c r="C9" s="1">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D9" s="1">
         <v>60</v>
@@ -986,7 +964,7 @@
         <v>30</v>
       </c>
       <c r="C11" s="1">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D11" s="1">
         <v>300</v>
@@ -1014,7 +992,7 @@
         <v>75</v>
       </c>
       <c r="C13" s="1">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D13" s="1">
         <v>150</v>
@@ -1028,7 +1006,7 @@
         <v>31</v>
       </c>
       <c r="C14" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D14" s="1">
         <v>150</v>
@@ -1084,7 +1062,7 @@
         <v>57</v>
       </c>
       <c r="C18" s="1">
-        <v>597</v>
+        <v>589</v>
       </c>
       <c r="D18" s="1">
         <v>70</v>
@@ -1284,6 +1262,31 @@
       </c>
       <c r="D32" s="1">
         <v>1100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DD5AD16-8BB8-496C-B2B6-80DA0CE31FAC}">
+  <sheetPr codeName="Hoja3"/>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cambios en la UI de la apk, ahora usa un menu desplegable y los paneles de estado se encuentran uno del lado del otro
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A293CDF-F465-49B2-A315-E9FAF627A9E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC9DDB99-990A-431F-8572-A520199443BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pendientes" sheetId="4" r:id="rId1"/>
     <sheet name="Productos" sheetId="1" r:id="rId2"/>
     <sheet name="Merma" sheetId="5" r:id="rId3"/>
+    <sheet name="Entrada" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="84">
   <si>
     <t>Código</t>
   </si>
@@ -278,6 +279,21 @@
   </si>
   <si>
     <t>Cantidad</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Cant Inicial</t>
+  </si>
+  <si>
+    <t>Precio Venta</t>
+  </si>
+  <si>
+    <t>Precio Costo</t>
+  </si>
+  <si>
+    <t>VERDADERO</t>
   </si>
 </sst>
 </file>
@@ -414,7 +430,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -463,11 +479,37 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C2CB94C0-D619-434A-A4B0-0D891E997B38}" name="Tabla3" displayName="Tabla3" ref="A1:C2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:C2" xr:uid="{C2CB94C0-D619-434A-A4B0-0D891E997B38}"/>
+  <autoFilter ref="A1:C2" xr:uid="{C2CB94C0-D619-434A-A4B0-0D891E997B38}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{F6BD4EA0-F565-4D2F-ADA2-8BC99D6A95A4}" name="Codigo"/>
     <tableColumn id="2" xr3:uid="{5A4E880C-CBFA-4386-ADF7-91899EDE0D07}" name="Nombre"/>
     <tableColumn id="3" xr3:uid="{BDD438F1-0115-4245-A313-92BAFF363974}" name="Cantidad"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5D0D9D21-CFBE-40B0-905F-9CEA9F018289}" name="Tabla4" displayName="Tabla4" ref="A1:F2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:F2" xr:uid="{5D0D9D21-CFBE-40B0-905F-9CEA9F018289}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{C9AA696F-7288-4911-8605-0369C64B5DF3}" name="Codigo"/>
+    <tableColumn id="2" xr3:uid="{43642E4C-2CFB-4937-BB18-1E41CE79C192}" name="Nombre"/>
+    <tableColumn id="3" xr3:uid="{5D6AE620-0A3C-45BF-8826-B45671388313}" name="Fecha"/>
+    <tableColumn id="4" xr3:uid="{AFA158CF-A341-4CB0-819C-B4F92F2AF323}" name="Cant Inicial"/>
+    <tableColumn id="5" xr3:uid="{BE484644-CD6B-4E41-B2EC-16A9F354C370}" name="Precio Venta"/>
+    <tableColumn id="6" xr3:uid="{8E92BF82-F26E-4805-AFCD-AAE2D1711EAC}" name="Precio Costo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -785,7 +827,9 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4"/>
+      <c r="A2" s="4">
+        <v>4614600000</v>
+      </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -794,7 +838,9 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="J2" s="4" t="s">
+        <v>83</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1295,4 +1341,43 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F5322B1-A0F9-4A2B-B4EF-2B5AE2033503}">
+  <sheetPr codeName="Hoja4"/>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="4" max="4" width="11.90625" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" customWidth="1"/>
+    <col min="6" max="6" width="13.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Paso 2: Comenzar la funcion de guardar el producto para que lo añada al stock y lo muestre listo para vender
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DAC5A08-18E4-4348-916B-0622CCED7B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27B733BE-B178-49A3-B673-44B87C4466A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
   <si>
     <t>Código</t>
   </si>
@@ -256,8 +256,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J4" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:J4" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J5" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+  <autoFilter ref="A1:J5" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -605,7 +605,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38113A1C-B25C-45F8-90F0-F3D668297EF0}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.453125" style="1" customWidth="1"/>
@@ -700,6 +700,22 @@
         <v>23</v>
       </c>
     </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>4614600000</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Implementacion de en APK para dar entrada a productos.
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB8C4891-EA4E-4EDC-BF46-A056F18D944E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB037171-66F9-42E3-BC88-52818433F25F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pendientes" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
   <si>
     <t>Código</t>
   </si>
@@ -113,13 +113,40 @@
     <t>Precio Costo</t>
   </si>
   <si>
-    <t>VERDADERO</t>
-  </si>
-  <si>
-    <t>Prueba</t>
-  </si>
-  <si>
-    <t>Prueba 2</t>
+    <t>prueba 1</t>
+  </si>
+  <si>
+    <t>prueba 2</t>
+  </si>
+  <si>
+    <t>Pr_00003</t>
+  </si>
+  <si>
+    <t>Prueba 3</t>
+  </si>
+  <si>
+    <t>Pr_00004</t>
+  </si>
+  <si>
+    <t>Prueba 4</t>
+  </si>
+  <si>
+    <t>Pr_00005</t>
+  </si>
+  <si>
+    <t>Producto 5</t>
+  </si>
+  <si>
+    <t>Pr_00006</t>
+  </si>
+  <si>
+    <t>Que pasa</t>
+  </si>
+  <si>
+    <t>Pr_00007</t>
+  </si>
+  <si>
+    <t>Jjjj</t>
   </si>
 </sst>
 </file>
@@ -256,8 +283,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J6" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:J6" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+  <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -605,7 +632,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38113A1C-B25C-45F8-90F0-F3D668297EF0}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.453125" style="1" customWidth="1"/>
@@ -653,9 +680,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
-        <v>4614600000</v>
-      </c>
+      <c r="A2" s="4"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -664,73 +689,7 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="4">
-        <v>4614600000</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="4">
-        <v>4614600000</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>4614600000</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="4">
-        <v>4614600000</v>
-      </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4" t="s">
-        <v>23</v>
-      </c>
+      <c r="J2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -743,7 +702,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -771,13 +730,13 @@
         <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1">
-        <v>100</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -785,13 +744,83 @@
         <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="1">
+        <v>18</v>
+      </c>
+      <c r="D3" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="1">
-        <v>150</v>
-      </c>
-      <c r="D3" s="1">
-        <v>50</v>
+      <c r="B4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="1">
+        <v>34</v>
+      </c>
+      <c r="D4" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="1">
+        <v>97</v>
+      </c>
+      <c r="D5" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="1">
+        <v>13</v>
+      </c>
+      <c r="D6" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="1">
+        <v>98</v>
+      </c>
+      <c r="D7" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="1">
+        <v>29</v>
+      </c>
+      <c r="D8" s="1">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implementada la opcion de ver las ventas agrupadas por facturas, filtradas por fecha. Tambien implementada la opcion de revertir una venta que aun no se haya sincronizado.
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB037171-66F9-42E3-BC88-52818433F25F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{106377A0-9F98-4956-90F0-CA048D8AD5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pendientes" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>Código</t>
   </si>
@@ -86,67 +86,40 @@
     <t>Procesado</t>
   </si>
   <si>
+    <t>Codigo</t>
+  </si>
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Cant Inicial</t>
+  </si>
+  <si>
+    <t>Precio Venta</t>
+  </si>
+  <si>
+    <t>Precio Costo</t>
+  </si>
+  <si>
+    <t>Pr_00002</t>
+  </si>
+  <si>
+    <t>Prueba 2</t>
+  </si>
+  <si>
     <t>Pr_00001</t>
   </si>
   <si>
-    <t>Pr_00002</t>
-  </si>
-  <si>
-    <t>Codigo</t>
-  </si>
-  <si>
-    <t>Nombre</t>
-  </si>
-  <si>
-    <t>Cantidad</t>
-  </si>
-  <si>
-    <t>Fecha</t>
-  </si>
-  <si>
-    <t>Cant Inicial</t>
-  </si>
-  <si>
-    <t>Precio Venta</t>
-  </si>
-  <si>
-    <t>Precio Costo</t>
-  </si>
-  <si>
-    <t>prueba 1</t>
-  </si>
-  <si>
-    <t>prueba 2</t>
-  </si>
-  <si>
-    <t>Pr_00003</t>
-  </si>
-  <si>
-    <t>Prueba 3</t>
-  </si>
-  <si>
-    <t>Pr_00004</t>
-  </si>
-  <si>
-    <t>Prueba 4</t>
-  </si>
-  <si>
-    <t>Pr_00005</t>
-  </si>
-  <si>
-    <t>Producto 5</t>
-  </si>
-  <si>
-    <t>Pr_00006</t>
-  </si>
-  <si>
-    <t>Que pasa</t>
-  </si>
-  <si>
-    <t>Pr_00007</t>
-  </si>
-  <si>
-    <t>Jjjj</t>
+    <t>Prueba 1</t>
+  </si>
+  <si>
+    <t>VERDADERO</t>
   </si>
 </sst>
 </file>
@@ -283,7 +256,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -680,7 +653,9 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4"/>
+      <c r="A2" s="4">
+        <v>4614800004</v>
+      </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -689,7 +664,9 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="J2" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -702,7 +679,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -727,100 +704,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C2" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D2" s="1">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C3" s="1">
-        <v>18</v>
+        <v>95</v>
       </c>
       <c r="D3" s="1">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="1">
-        <v>34</v>
-      </c>
-      <c r="D4" s="1">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="1">
-        <v>97</v>
-      </c>
-      <c r="D5" s="1">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="1">
-        <v>13</v>
-      </c>
-      <c r="D6" s="1">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="1">
-        <v>98</v>
-      </c>
-      <c r="D7" s="1">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="1">
-        <v>29</v>
-      </c>
-      <c r="D8" s="1">
-        <v>48</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -839,13 +746,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
         <v>16</v>
-      </c>
-      <c r="B1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -869,22 +776,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>20</v>
-      </c>
-      <c r="E1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Paso 2: Quedo lista la funcion de abastecimiento desde la app hasta datos.xlsx
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{106377A0-9F98-4956-90F0-CA048D8AD5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110C2952-B38B-420A-A8F0-0A03935D6464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="Productos" sheetId="1" r:id="rId2"/>
     <sheet name="Merma" sheetId="5" r:id="rId3"/>
     <sheet name="Entrada" sheetId="6" r:id="rId4"/>
+    <sheet name="Abastecimiento" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
   <si>
     <t>Código</t>
   </si>
@@ -107,19 +108,22 @@
     <t>Precio Costo</t>
   </si>
   <si>
+    <t>Pr_00001</t>
+  </si>
+  <si>
+    <t>Prueba 1</t>
+  </si>
+  <si>
     <t>Pr_00002</t>
   </si>
   <si>
     <t>Prueba 2</t>
   </si>
   <si>
-    <t>Pr_00001</t>
-  </si>
-  <si>
-    <t>Prueba 1</t>
-  </si>
-  <si>
-    <t>VERDADERO</t>
+    <t>2026-05-07T03:16:35.565Z</t>
+  </si>
+  <si>
+    <t>2026-05-07T03:16:45.921Z</t>
   </si>
 </sst>
 </file>
@@ -256,7 +260,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -653,9 +657,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
-        <v>4614800004</v>
-      </c>
+      <c r="A2" s="4"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -664,9 +666,7 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="J2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -704,30 +704,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="D2" s="1">
-        <v>10</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C3" s="1">
-        <v>95</v>
+        <v>200</v>
       </c>
       <c r="D3" s="1">
-        <v>250</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -800,4 +800,47 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AA63D08-2BDB-4554-A815-29AFCF757F0F}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Se quita el panel de debug innecesario en el frontend
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110C2952-B38B-420A-A8F0-0A03935D6464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{471C933E-E275-43DD-B5C8-6ADBC6D28DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pendientes" sheetId="4" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>Código</t>
   </si>
@@ -111,19 +111,25 @@
     <t>Pr_00001</t>
   </si>
   <si>
+    <t>Pr_00002</t>
+  </si>
+  <si>
     <t>Prueba 1</t>
   </si>
   <si>
-    <t>Pr_00002</t>
-  </si>
-  <si>
     <t>Prueba 2</t>
   </si>
   <si>
-    <t>2026-05-07T03:16:35.565Z</t>
-  </si>
-  <si>
-    <t>2026-05-07T03:16:45.921Z</t>
+    <t>Pr_00003</t>
+  </si>
+  <si>
+    <t>Prueba 3</t>
+  </si>
+  <si>
+    <t>Pr_00004</t>
+  </si>
+  <si>
+    <t>Prueba 4</t>
   </si>
 </sst>
 </file>
@@ -679,7 +685,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -707,7 +713,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1">
         <v>100</v>
@@ -718,7 +724,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>24</v>
@@ -728,6 +734,34 @@
       </c>
       <c r="D3" s="1">
         <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="1">
+        <v>300</v>
+      </c>
+      <c r="D4" s="1">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="1">
+        <v>400</v>
+      </c>
+      <c r="D5" s="1">
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -804,7 +838,8 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AA63D08-2BDB-4554-A815-29AFCF757F0F}">
-  <dimension ref="A1:C3"/>
+  <sheetPr codeName="Hoja5"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -818,28 +853,6 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadida la funcionalidad de añadir gastos variables desde la apk.
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{471C933E-E275-43DD-B5C8-6ADBC6D28DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB9712E-58B7-42F8-BFFD-B3E93E5064DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pendientes" sheetId="4" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Merma" sheetId="5" r:id="rId3"/>
     <sheet name="Entrada" sheetId="6" r:id="rId4"/>
     <sheet name="Abastecimiento" sheetId="7" r:id="rId5"/>
+    <sheet name="Gastos" sheetId="8" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
   <si>
     <t>Código</t>
   </si>
@@ -108,28 +109,31 @@
     <t>Precio Costo</t>
   </si>
   <si>
+    <t>Descripcion</t>
+  </si>
+  <si>
+    <t>Monto</t>
+  </si>
+  <si>
     <t>Pr_00001</t>
   </si>
   <si>
     <t>Pr_00002</t>
   </si>
   <si>
-    <t>Prueba 1</t>
-  </si>
-  <si>
-    <t>Prueba 2</t>
+    <t>aceite</t>
+  </si>
+  <si>
+    <t>Chicharo</t>
   </si>
   <si>
     <t>Pr_00003</t>
   </si>
   <si>
-    <t>Prueba 3</t>
-  </si>
-  <si>
-    <t>Pr_00004</t>
-  </si>
-  <si>
-    <t>Prueba 4</t>
+    <t>Sal</t>
+  </si>
+  <si>
+    <t>VERDADERO</t>
   </si>
 </sst>
 </file>
@@ -266,7 +270,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -663,7 +667,9 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4"/>
+      <c r="A2" s="4">
+        <v>4615700000</v>
+      </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -672,7 +678,9 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="J2" s="4" t="s">
+        <v>29</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -685,7 +693,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -710,58 +718,44 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C2" s="1">
-        <v>100</v>
+        <v>168</v>
       </c>
       <c r="D2" s="1">
-        <v>100</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C3" s="1">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D3" s="1">
-        <v>200</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C4" s="1">
-        <v>300</v>
+        <v>696</v>
       </c>
       <c r="D4" s="1">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="1">
-        <v>400</v>
-      </c>
-      <c r="D5" s="1">
-        <v>400</v>
+        <v>700</v>
       </c>
     </row>
   </sheetData>
@@ -856,4 +850,26 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C810362F-EE1A-4FB4-B169-9E00B4792D8D}">
+  <sheetPr codeName="Hoja6"/>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Incluido desglose de pendientes de forma desplegable y añadida visibilidad de los gastos variables en el resumen del dia
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB9712E-58B7-42F8-BFFD-B3E93E5064DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{710C80C5-9238-47B3-8B43-C43E42D12435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
   <si>
     <t>Código</t>
   </si>
@@ -270,8 +270,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J3" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+  <autoFilter ref="A1:J3" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -619,7 +619,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38113A1C-B25C-45F8-90F0-F3D668297EF0}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.453125" style="1" customWidth="1"/>
@@ -682,6 +682,22 @@
         <v>29</v>
       </c>
     </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>4615800000</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Reorganizacion de Gestion Plus
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{710C80C5-9238-47B3-8B43-C43E42D12435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CAF790C-2C5A-4999-B468-E11914DDFAA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
   <si>
     <t>Código</t>
   </si>
@@ -115,22 +115,16 @@
     <t>Monto</t>
   </si>
   <si>
-    <t>Pr_00001</t>
-  </si>
-  <si>
     <t>Pr_00002</t>
   </si>
   <si>
-    <t>aceite</t>
-  </si>
-  <si>
-    <t>Chicharo</t>
-  </si>
-  <si>
     <t>Pr_00003</t>
   </si>
   <si>
-    <t>Sal</t>
+    <t>Arepa</t>
+  </si>
+  <si>
+    <t>Arepa grande</t>
   </si>
   <si>
     <t>VERDADERO</t>
@@ -270,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J3" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:J3" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J4" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+  <autoFilter ref="A1:J4" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -619,7 +613,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38113A1C-B25C-45F8-90F0-F3D668297EF0}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.453125" style="1" customWidth="1"/>
@@ -668,7 +662,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>4615700000</v>
+        <v>4616800001</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -679,12 +673,12 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
-        <v>4615800000</v>
+        <v>4616800001</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -695,7 +689,23 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>4616800001</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -709,7 +719,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -740,10 +750,10 @@
         <v>25</v>
       </c>
       <c r="C2" s="1">
-        <v>168</v>
+        <v>100</v>
       </c>
       <c r="D2" s="1">
-        <v>1000</v>
+        <v>40.037349999999996</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -754,24 +764,10 @@
         <v>26</v>
       </c>
       <c r="C3" s="1">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D3" s="1">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" s="1">
-        <v>696</v>
-      </c>
-      <c r="D4" s="1">
-        <v>700</v>
+        <v>80.074699999999993</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Arreglado un bug de escritura en datos.xlsx y solucionado perdida de datos si varias app sincronizan datos a la vez
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F495BEEA-08A2-463F-84E4-BC6CD77DB1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C3C44DF-D965-4C41-A866-47DD70D73E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
   <si>
     <t>Código</t>
   </si>
@@ -115,19 +115,10 @@
     <t>Monto</t>
   </si>
   <si>
-    <t>Pr_00002</t>
-  </si>
-  <si>
-    <t>Pr_00003</t>
-  </si>
-  <si>
-    <t>Arepa</t>
-  </si>
-  <si>
-    <t>Arepa grande</t>
-  </si>
-  <si>
-    <t>VERDADERO</t>
+    <t>Pr_00001</t>
+  </si>
+  <si>
+    <t>Cable m</t>
   </si>
 </sst>
 </file>
@@ -264,8 +255,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J5" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:J5" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+  <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -613,7 +604,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38113A1C-B25C-45F8-90F0-F3D668297EF0}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.453125" style="1" customWidth="1"/>
@@ -661,9 +652,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
-        <v>4616800001</v>
-      </c>
+      <c r="A2" s="4"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -672,57 +661,7 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="4">
-        <v>4616800001</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="4">
-        <v>4616800001</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>4616800000</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="J2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -735,7 +674,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -763,27 +702,13 @@
         <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" s="1">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="D2" s="1">
-        <v>40.037349999999996</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="1">
-        <v>200</v>
-      </c>
-      <c r="D3" s="1">
-        <v>80.074699999999993</v>
+        <v>1500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mejora en la consistencia de la concurrencia y arreglado par de errores
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C3C44DF-D965-4C41-A866-47DD70D73E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C07D0D-1F58-4384-96AD-39F87390F318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
   <si>
     <t>Código</t>
   </si>
@@ -119,6 +119,12 @@
   </si>
   <si>
     <t>Cable m</t>
+  </si>
+  <si>
+    <t>Pr_00002</t>
+  </si>
+  <si>
+    <t>Breaker</t>
   </si>
 </sst>
 </file>
@@ -674,7 +680,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -705,10 +711,24 @@
         <v>24</v>
       </c>
       <c r="C2" s="1">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D2" s="1">
         <v>1500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="1">
+        <v>7</v>
+      </c>
+      <c r="D3" s="1">
+        <v>3500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Establecido todo lo necesario para el manejo de concurrencias. Cada vez que el servidor va a escribir en datos.xlsx revisa que no hayan duplicados y si los hay mapea todo a un nuevo ID
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C07D0D-1F58-4384-96AD-39F87390F318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{398CC684-0BDF-454F-AFA6-FF17938B1968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
   <si>
     <t>Código</t>
   </si>
@@ -125,6 +125,30 @@
   </si>
   <si>
     <t>Breaker</t>
+  </si>
+  <si>
+    <t>Pr_00003</t>
+  </si>
+  <si>
+    <t>Losas</t>
+  </si>
+  <si>
+    <t>Pr_00004</t>
+  </si>
+  <si>
+    <t>Escobas</t>
+  </si>
+  <si>
+    <t>Pr_00005</t>
+  </si>
+  <si>
+    <t>Pelotas</t>
+  </si>
+  <si>
+    <t>Pr_00006</t>
+  </si>
+  <si>
+    <t>Tijeras</t>
   </si>
 </sst>
 </file>
@@ -680,7 +704,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -705,30 +729,86 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1">
-        <v>90</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1">
-        <v>1500</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C3" s="1">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="D3" s="1">
-        <v>3500</v>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="1">
+        <v>20</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="1">
+        <v>20</v>
+      </c>
+      <c r="D5" s="1">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="1">
+        <v>90</v>
+      </c>
+      <c r="D6" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="1">
+        <v>30</v>
+      </c>
+      <c r="D7" s="1">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
some changes in UX and UI
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{398CC684-0BDF-454F-AFA6-FF17938B1968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74BE6CFE-2AB1-46AB-BFF6-FCC721477979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
   <si>
     <t>Código</t>
   </si>
@@ -118,37 +118,13 @@
     <t>Pr_00001</t>
   </si>
   <si>
-    <t>Cable m</t>
-  </si>
-  <si>
     <t>Pr_00002</t>
   </si>
   <si>
-    <t>Breaker</t>
-  </si>
-  <si>
-    <t>Pr_00003</t>
-  </si>
-  <si>
-    <t>Losas</t>
-  </si>
-  <si>
-    <t>Pr_00004</t>
-  </si>
-  <si>
-    <t>Escobas</t>
-  </si>
-  <si>
-    <t>Pr_00005</t>
-  </si>
-  <si>
-    <t>Pelotas</t>
-  </si>
-  <si>
-    <t>Pr_00006</t>
-  </si>
-  <si>
-    <t>Tijeras</t>
+    <t>VERDADERO</t>
+  </si>
+  <si>
+    <t>Arepa</t>
   </si>
 </sst>
 </file>
@@ -285,7 +261,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -682,7 +658,9 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4"/>
+      <c r="A2" s="4">
+        <v>4617300001</v>
+      </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -691,7 +669,9 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="J2" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -704,7 +684,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -729,86 +709,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C2" s="1">
-        <v>7</v>
+        <v>140</v>
       </c>
       <c r="D2" s="1">
-        <v>3500</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C3" s="1">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="D3" s="1">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="1">
-        <v>20</v>
-      </c>
-      <c r="D4" s="1">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="1">
-        <v>20</v>
-      </c>
-      <c r="D5" s="1">
-        <v>4500</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="1">
-        <v>90</v>
-      </c>
-      <c r="D6" s="1">
         <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="1">
-        <v>30</v>
-      </c>
-      <c r="D7" s="1">
-        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Añadida toda la logica que permite procesar elaboraciones de productos desde la app.
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74BE6CFE-2AB1-46AB-BFF6-FCC721477979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E601D1-BC72-4727-AF8E-9D27AA6A4B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pendientes" sheetId="4" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="Entrada" sheetId="6" r:id="rId4"/>
     <sheet name="Abastecimiento" sheetId="7" r:id="rId5"/>
     <sheet name="Gastos" sheetId="8" r:id="rId6"/>
+    <sheet name="Elaboracion" sheetId="9" r:id="rId7"/>
+    <sheet name="Recetas" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
   <si>
     <t>Código</t>
   </si>
@@ -115,16 +117,28 @@
     <t>Monto</t>
   </si>
   <si>
+    <t>Arepa</t>
+  </si>
+  <si>
+    <t>CantLote</t>
+  </si>
+  <si>
+    <t>PrecioVenta</t>
+  </si>
+  <si>
+    <t>Lotes</t>
+  </si>
+  <si>
+    <t>PrecioCosto</t>
+  </si>
+  <si>
+    <t>NombreReceta</t>
+  </si>
+  <si>
     <t>Pr_00001</t>
   </si>
   <si>
     <t>Pr_00002</t>
-  </si>
-  <si>
-    <t>VERDADERO</t>
-  </si>
-  <si>
-    <t>Arepa</t>
   </si>
 </sst>
 </file>
@@ -261,7 +275,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -291,8 +305,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F16977D9-4AF0-4513-B527-4EA8B61A33F3}" name="ALMACEN" displayName="ALMACEN" ref="A1:D33" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4" headerRowCellStyle="Énfasis5">
-  <autoFilter ref="A1:D33" xr:uid="{F16977D9-4AF0-4513-B527-4EA8B61A33F3}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F16977D9-4AF0-4513-B527-4EA8B61A33F3}" name="ALMACEN" displayName="ALMACEN" ref="A1:D31" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4" headerRowCellStyle="Énfasis5">
+  <autoFilter ref="A1:D31" xr:uid="{F16977D9-4AF0-4513-B527-4EA8B61A33F3}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -658,9 +672,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
-        <v>4617300001</v>
-      </c>
+      <c r="A2" s="4"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -669,9 +681,7 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="J2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -709,13 +719,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>140</v>
+        <v>10</v>
       </c>
       <c r="D2" s="1">
         <v>100</v>
@@ -723,16 +733,16 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C3" s="1">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -849,4 +859,65 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46499A14-3E78-4305-81DD-11F1CA3E065C}">
+  <sheetPr codeName="Hoja7"/>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{613846D1-0EB6-4FE0-98B3-AC7E9DC64E9C}">
+  <sheetPr codeName="Hoja8"/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <v>50</v>
+      </c>
+      <c r="D2">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ahora se ven tambien los ingredientes necesarios al elaborar en la app.
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E601D1-BC72-4727-AF8E-9D27AA6A4B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{886D6AF8-00C9-4200-ABF1-DD50DED34D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pendientes" sheetId="4" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="43">
   <si>
     <t>Código</t>
   </si>
@@ -139,6 +139,42 @@
   </si>
   <si>
     <t>Pr_00002</t>
+  </si>
+  <si>
+    <t>Ingredientes</t>
+  </si>
+  <si>
+    <t>Receta</t>
+  </si>
+  <si>
+    <t>Unidad</t>
+  </si>
+  <si>
+    <t>Azucar</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>Harina</t>
+  </si>
+  <si>
+    <t>Pr_00003</t>
+  </si>
+  <si>
+    <t>Prueba</t>
+  </si>
+  <si>
+    <t>Pr_00004</t>
+  </si>
+  <si>
+    <t>Toallas</t>
+  </si>
+  <si>
+    <t>Pr_00005</t>
+  </si>
+  <si>
+    <t>Prueba 2</t>
   </si>
 </sst>
 </file>
@@ -694,7 +730,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -725,7 +761,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1">
         <v>100</v>
@@ -739,10 +775,52 @@
         <v>23</v>
       </c>
       <c r="C3" s="1">
-        <v>20</v>
+        <v>106</v>
       </c>
       <c r="D3" s="1">
         <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1005</v>
+      </c>
+      <c r="D5" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="1">
+        <v>21</v>
+      </c>
+      <c r="D6" s="1">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -864,7 +942,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46499A14-3E78-4305-81DD-11F1CA3E065C}">
   <sheetPr codeName="Hoja7"/>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
@@ -878,6 +956,14 @@
         <v>26</v>
       </c>
     </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -886,10 +972,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{613846D1-0EB6-4FE0-98B3-AC7E9DC64E9C}">
   <sheetPr codeName="Hoja8"/>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -902,8 +988,20 @@
       <c r="D1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="F1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -915,6 +1013,32 @@
       </c>
       <c r="D2">
         <v>20</v>
+      </c>
+      <c r="F2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix sobre inconsistencias del funcionamiento SqLite de la apk.
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{886D6AF8-00C9-4200-ABF1-DD50DED34D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{559EB9EA-40C4-4209-B379-6291B5F6035B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="46">
   <si>
     <t>Código</t>
   </si>
@@ -175,6 +175,15 @@
   </si>
   <si>
     <t>Prueba 2</t>
+  </si>
+  <si>
+    <t>Pr_00006</t>
+  </si>
+  <si>
+    <t>Pr_00007</t>
+  </si>
+  <si>
+    <t>Joyas</t>
   </si>
 </sst>
 </file>
@@ -730,7 +739,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -761,7 +770,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D2" s="1">
         <v>100</v>
@@ -775,7 +784,7 @@
         <v>23</v>
       </c>
       <c r="C3" s="1">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D3" s="1">
         <v>50</v>
@@ -789,7 +798,7 @@
         <v>38</v>
       </c>
       <c r="C4" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D4" s="1">
         <v>100</v>
@@ -803,7 +812,7 @@
         <v>40</v>
       </c>
       <c r="C5" s="1">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="D5" s="1">
         <v>50</v>
@@ -817,10 +826,38 @@
         <v>42</v>
       </c>
       <c r="C6" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D6" s="1">
         <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="1">
+        <v>20</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="1">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1">
+        <v>5000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mejora en la UX durante el escaneo automatico del IP del servidor, mejora en la optimizacion y eficiencia del escaneo. Arreglado que no se tomaba la ultima factura desde el excel hacia la app como referencia cuando no habian datos pendientes.
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{559EB9EA-40C4-4209-B379-6291B5F6035B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40131310-89E6-4066-A922-FE85064AF380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
   <si>
     <t>Código</t>
   </si>
@@ -184,6 +184,15 @@
   </si>
   <si>
     <t>Joyas</t>
+  </si>
+  <si>
+    <t>Pr_00008</t>
+  </si>
+  <si>
+    <t>Ollas</t>
+  </si>
+  <si>
+    <t>VERDADERO</t>
   </si>
 </sst>
 </file>
@@ -320,7 +329,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -717,7 +726,9 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4"/>
+      <c r="A2" s="4">
+        <v>4617600003</v>
+      </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -726,7 +737,9 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="J2" s="4" t="s">
+        <v>48</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -739,7 +752,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -770,7 +783,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D2" s="1">
         <v>100</v>
@@ -784,7 +797,7 @@
         <v>23</v>
       </c>
       <c r="C3" s="1">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D3" s="1">
         <v>50</v>
@@ -812,7 +825,7 @@
         <v>40</v>
       </c>
       <c r="C5" s="1">
-        <v>1004</v>
+        <v>984</v>
       </c>
       <c r="D5" s="1">
         <v>50</v>
@@ -854,10 +867,24 @@
         <v>45</v>
       </c>
       <c r="C8" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D8" s="1">
         <v>5000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="1">
+        <v>8</v>
+      </c>
+      <c r="D9" s="1">
+        <v>35000</v>
       </c>
     </row>
   </sheetData>
@@ -979,7 +1006,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46499A14-3E78-4305-81DD-11F1CA3E065C}">
   <sheetPr codeName="Hoja7"/>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
@@ -991,14 +1018,6 @@
       </c>
       <c r="B1" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1043,13 +1062,13 @@
         <v>23</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="C2">
         <v>50</v>
       </c>
       <c r="D2">
-        <v>20</v>
+        <v>15.981</v>
       </c>
       <c r="F2" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Edge case solucionado de conflicto con IDs de factura y un poco de depuracion del codigo
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40131310-89E6-4066-A922-FE85064AF380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775C1594-BEF4-4E97-95D5-F7968DC5EDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="50">
   <si>
     <t>Código</t>
   </si>
@@ -159,40 +159,43 @@
     <t>Harina</t>
   </si>
   <si>
-    <t>Pr_00003</t>
+    <t>Pr_00004</t>
+  </si>
+  <si>
+    <t>Toallas</t>
+  </si>
+  <si>
+    <t>Pr_00005</t>
+  </si>
+  <si>
+    <t>Prueba 2</t>
+  </si>
+  <si>
+    <t>Pr_00006</t>
+  </si>
+  <si>
+    <t>Pr_00007</t>
+  </si>
+  <si>
+    <t>Joyas</t>
+  </si>
+  <si>
+    <t>Pr_00008</t>
+  </si>
+  <si>
+    <t>Ollas</t>
+  </si>
+  <si>
+    <t>Pr_00009</t>
+  </si>
+  <si>
+    <t>Aceite</t>
+  </si>
+  <si>
+    <t>Pr_00010</t>
   </si>
   <si>
     <t>Prueba</t>
-  </si>
-  <si>
-    <t>Pr_00004</t>
-  </si>
-  <si>
-    <t>Toallas</t>
-  </si>
-  <si>
-    <t>Pr_00005</t>
-  </si>
-  <si>
-    <t>Prueba 2</t>
-  </si>
-  <si>
-    <t>Pr_00006</t>
-  </si>
-  <si>
-    <t>Pr_00007</t>
-  </si>
-  <si>
-    <t>Joyas</t>
-  </si>
-  <si>
-    <t>Pr_00008</t>
-  </si>
-  <si>
-    <t>Ollas</t>
-  </si>
-  <si>
-    <t>VERDADERO</t>
   </si>
 </sst>
 </file>
@@ -329,7 +332,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}" name="Tabla1" displayName="Tabla1" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:J2" xr:uid="{BF1E74FB-25A2-4E5C-B6A5-8A3881088760}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -726,9 +729,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
-        <v>4617600003</v>
-      </c>
+      <c r="A2" s="4"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -737,9 +738,7 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4" t="s">
-        <v>48</v>
-      </c>
+      <c r="J2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -752,7 +751,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
@@ -783,7 +782,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D2" s="1">
         <v>100</v>
@@ -797,7 +796,7 @@
         <v>23</v>
       </c>
       <c r="C3" s="1">
-        <v>114</v>
+        <v>302</v>
       </c>
       <c r="D3" s="1">
         <v>50</v>
@@ -811,10 +810,10 @@
         <v>38</v>
       </c>
       <c r="C4" s="1">
-        <v>0</v>
+        <v>969</v>
       </c>
       <c r="D4" s="1">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -825,10 +824,10 @@
         <v>40</v>
       </c>
       <c r="C5" s="1">
-        <v>984</v>
+        <v>20</v>
       </c>
       <c r="D5" s="1">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -836,27 +835,27 @@
         <v>41</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C6" s="1">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="C7" s="1">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D7" s="1">
-        <v>1000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -870,7 +869,7 @@
         <v>7</v>
       </c>
       <c r="D8" s="1">
-        <v>5000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -881,10 +880,24 @@
         <v>47</v>
       </c>
       <c r="C9" s="1">
-        <v>8</v>
+        <v>150</v>
       </c>
       <c r="D9" s="1">
-        <v>35000</v>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="1">
+        <v>100</v>
+      </c>
+      <c r="D10" s="1">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mas depuracion del codigo
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775C1594-BEF4-4E97-95D5-F7968DC5EDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A4DB8E-F716-471E-9E01-ECD18634F594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -782,7 +782,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D2" s="1">
         <v>100</v>
@@ -796,7 +796,7 @@
         <v>23</v>
       </c>
       <c r="C3" s="1">
-        <v>302</v>
+        <v>400</v>
       </c>
       <c r="D3" s="1">
         <v>50</v>
@@ -810,7 +810,7 @@
         <v>38</v>
       </c>
       <c r="C4" s="1">
-        <v>969</v>
+        <v>962</v>
       </c>
       <c r="D4" s="1">
         <v>50</v>
@@ -824,7 +824,7 @@
         <v>40</v>
       </c>
       <c r="C5" s="1">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D5" s="1">
         <v>10</v>
@@ -880,7 +880,7 @@
         <v>47</v>
       </c>
       <c r="C9" s="1">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D9" s="1">
         <v>1500</v>
@@ -894,7 +894,7 @@
         <v>49</v>
       </c>
       <c r="C10" s="1">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D10" s="1">
         <v>100</v>

</xml_diff>